<commit_message>
Prefer Shopify shop money for refunds
</commit_message>
<xml_diff>
--- a/output/spreadsheet/pyg_sl_2026.xlsx
+++ b/output/spreadsheet/pyg_sl_2026.xlsx
@@ -868,7 +868,7 @@
     <row r="3" ht="12" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Shopify daily average | Actualizado: 10/08/2026 23:59 h</t>
+          <t>Shopify daily average | Actualizado: 11/08/2026 00:13 h</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -19616,7 +19616,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-10T21:59:52Z</t>
+          <t>2026-08-10T22:13:48Z</t>
         </is>
       </c>
     </row>
@@ -23574,7 +23574,7 @@
         </is>
       </c>
       <c r="E82" s="50" t="n">
-        <v>19210.62</v>
+        <v>792.85</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -23590,7 +23590,7 @@
         <v>1</v>
       </c>
       <c r="I82" s="50" t="n">
-        <v>19210.62</v>
+        <v>792.85</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -23670,7 +23670,7 @@
         </is>
       </c>
       <c r="E84" s="50" t="n">
-        <v>13571.05</v>
+        <v>1737.85</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -23686,7 +23686,7 @@
         <v>1</v>
       </c>
       <c r="I84" s="50" t="n">
-        <v>13571.05</v>
+        <v>1737.85</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -23910,7 +23910,7 @@
         </is>
       </c>
       <c r="E89" s="50" t="n">
-        <v>11435.23</v>
+        <v>2595.85</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -23926,7 +23926,7 @@
         <v>1</v>
       </c>
       <c r="I89" s="50" t="n">
-        <v>11435.23</v>
+        <v>2595.85</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
@@ -24006,7 +24006,7 @@
         </is>
       </c>
       <c r="E91" s="50" t="n">
-        <v>17609.98</v>
+        <v>1606.98</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -24022,7 +24022,7 @@
         <v>1</v>
       </c>
       <c r="I91" s="50" t="n">
-        <v>17609.98</v>
+        <v>1606.98</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>

</xml_diff>